<commit_message>
Creacion cruds jornadas y tipo de rama
</commit_message>
<xml_diff>
--- a/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
+++ b/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
@@ -16,7 +16,7 @@
     <t>Reporte de Resultados de Pruebas Automatizadas</t>
   </si>
   <si>
-    <t>Generado: 25/3/2026, 10:46:25</t>
+    <t>Generado: 25/3/2026, 15:46:36</t>
   </si>
   <si>
     <t>No de prueba</t>
@@ -37,10 +37,10 @@
     <t>Evidencia</t>
   </si>
   <si>
-    <t>Paises que la usan</t>
-  </si>
-  <si>
-    <t>Moneda: GTQ - Pais: Guatemala</t>
+    <t>Tipo agencia o rama</t>
+  </si>
+  <si>
+    <t>Código: 2 - Nombre: Sucursal</t>
   </si>
   <si>
     <t>exitosa</t>
@@ -49,13 +49,13 @@
     <t>El registro se ha guardado correctamente</t>
   </si>
   <si>
-    <t>Captura-1-Moneda &gt; Paises que la usan-exitosa.png</t>
-  </si>
-  <si>
-    <t>Moneda: L - Pais: Honduras TR</t>
-  </si>
-  <si>
-    <t>Captura-2-Moneda &gt; Paises que la usan-exitosa.png</t>
+    <t>Captura-1-Tipo agencia o rama-exitosa.png</t>
+  </si>
+  <si>
+    <t>Código: 3 - Nombre: Ventanilla</t>
+  </si>
+  <si>
+    <t>Captura-2-Tipo agencia o rama-exitosa.png</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
valores globales y tarea para eliminar capturas
</commit_message>
<xml_diff>
--- a/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
+++ b/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>Reporte de Resultados de Pruebas Automatizadas</t>
   </si>
   <si>
-    <t>Generado: 25/3/2026, 9:34:13</t>
+    <t>Generado: 25/3/2026, 15:47:45</t>
   </si>
   <si>
     <t>No de prueba</t>
@@ -37,22 +37,25 @@
     <t>Evidencia</t>
   </si>
   <si>
-    <t>Denominación</t>
-  </si>
-  <si>
-    <t>Moneda: L - Nombre: 1 Lempira - Monto: 1</t>
-  </si>
-  <si>
-    <t>exitosa</t>
-  </si>
-  <si>
-    <t>El registro se ha guardado correctamente</t>
-  </si>
-  <si>
-    <t>Captura-2-Denominacion-exitosa.png</t>
-  </si>
-  <si>
-    <t>Moneda: L - Nombre: 2 Lempiras - Monto: 2</t>
+    <t>Valores Globales</t>
+  </si>
+  <si>
+    <t>Código: 3312 - Tipo: Numérico</t>
+  </si>
+  <si>
+    <t>fallida</t>
+  </si>
+  <si>
+    <t>CASTV-0181 - Error. Ya existe un registro con el mismo código de valor global.</t>
+  </si>
+  <si>
+    <t>Captura-1-Valores Globales-fallida.png</t>
+  </si>
+  <si>
+    <t>Código: 3321 - Tipo: Alfanumérico</t>
+  </si>
+  <si>
+    <t>Captura-2-Valores Globales-fallida.png</t>
   </si>
 </sst>
 </file>
@@ -515,7 +518,7 @@
     <col min="2" max="2" width="27" customWidth="1"/>
     <col min="3" max="3" width="52" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
+    <col min="5" max="5" width="80" customWidth="1"/>
     <col min="6" max="6" width="52" customWidth="1"/>
   </cols>
   <sheetData>
@@ -555,7 +558,7 @@
     </row>
     <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>8</v>
@@ -590,7 +593,7 @@
         <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
division geografica 3er sub nivel
</commit_message>
<xml_diff>
--- a/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
+++ b/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Reporte de Resultados de Pruebas Automatizadas</t>
   </si>
   <si>
-    <t>Generado: 25/3/2026, 17:52:45</t>
+    <t>Generado: 25/3/2026, 19:33:48</t>
   </si>
   <si>
     <t>No de prueba</t>
@@ -35,39 +35,6 @@
   </si>
   <si>
     <t>Evidencia</t>
-  </si>
-  <si>
-    <t>Nivel De Autorizacion</t>
-  </si>
-  <si>
-    <t>Arbol: Byte S.A. - Nivel: 0 - Nombre: nombre QA-Auto 1</t>
-  </si>
-  <si>
-    <t>exitosa</t>
-  </si>
-  <si>
-    <t>El registro se ha guardado correctamente</t>
-  </si>
-  <si>
-    <t>Captura-1-Nivel De Autorizacion-exitosa.png</t>
-  </si>
-  <si>
-    <t>Arbol: Byte S.A. - Nivel: 1 - Nombre: nombre QA-Auto 2</t>
-  </si>
-  <si>
-    <t>fallida</t>
-  </si>
-  <si>
-    <t>CASTV-0217 - Error. Ya existe un registro con el mismo nivel.</t>
-  </si>
-  <si>
-    <t>Captura-2-Nivel De Autorizacion-fallida.png</t>
-  </si>
-  <si>
-    <t>Arbol: Byte S.A. - Nivel: 2 - Nombre: nombre QA-Auto 3</t>
-  </si>
-  <si>
-    <t>Captura-3-Nivel De Autorizacion-fallida.png</t>
   </si>
 </sst>
 </file>
@@ -98,7 +65,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -108,11 +75,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0070C0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -128,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -139,7 +101,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -523,14 +484,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:F8"/>
+  <dimension ref="A2:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
-    <col min="3" max="3" width="56" customWidth="1"/>
+    <col min="3" max="3" width="52" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="63" customWidth="1"/>
+    <col min="5" max="5" width="42" customWidth="1"/>
     <col min="6" max="6" width="52" customWidth="1"/>
   </cols>
   <sheetData>
@@ -566,66 +527,6 @@
       </c>
       <c r="F5" s="3" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
-        <v>1</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>2</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4">
-        <v>3</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
departamentos y parametros generales
</commit_message>
<xml_diff>
--- a/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
+++ b/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>Reporte de Resultados de Pruebas Automatizadas</t>
   </si>
   <si>
-    <t>Generado: 25/3/2026, 19:33:48</t>
+    <t>Generado: 25/3/2026, 19:56:54</t>
   </si>
   <si>
     <t>No de prueba</t>
@@ -35,6 +35,27 @@
   </si>
   <si>
     <t>Evidencia</t>
+  </si>
+  <si>
+    <t>Departamentos</t>
+  </si>
+  <si>
+    <t>Código: 1 - Nombre: Departamento QA-Auto 1</t>
+  </si>
+  <si>
+    <t>fallida</t>
+  </si>
+  <si>
+    <t>CASTV-0097 - Error.Ya existe un registro con el mismo código de departamento.</t>
+  </si>
+  <si>
+    <t>Captura-1-Departamentos-fallida.png</t>
+  </si>
+  <si>
+    <t>Código: 2 - Nombre: Departamento QA-Auto 2</t>
+  </si>
+  <si>
+    <t>Captura-2-Departamentos-fallida.png</t>
   </si>
 </sst>
 </file>
@@ -65,7 +86,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -75,6 +96,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0070C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -101,6 +127,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -484,14 +511,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:F5"/>
+  <dimension ref="A2:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
     <col min="3" max="3" width="52" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
+    <col min="5" max="5" width="79" customWidth="1"/>
     <col min="6" max="6" width="52" customWidth="1"/>
   </cols>
   <sheetData>
@@ -527,6 +554,46 @@
       </c>
       <c r="F5" s="3" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>1</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
arbol organizacional y metodo llenarcampoIframe mejorado(cuando existe mas de un selector visible le da 10 puntos mas al que es visible, pendiente asignar las transacciones)
</commit_message>
<xml_diff>
--- a/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
+++ b/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Reporte de Resultados de Pruebas Automatizadas</t>
   </si>
   <si>
-    <t>Generado: 25/3/2026, 19:56:54</t>
+    <t>Generado: 26/3/2026, 14:32:28</t>
   </si>
   <si>
     <t>No de prueba</t>
@@ -35,27 +35,6 @@
   </si>
   <si>
     <t>Evidencia</t>
-  </si>
-  <si>
-    <t>Departamentos</t>
-  </si>
-  <si>
-    <t>Código: 1 - Nombre: Departamento QA-Auto 1</t>
-  </si>
-  <si>
-    <t>fallida</t>
-  </si>
-  <si>
-    <t>CASTV-0097 - Error.Ya existe un registro con el mismo código de departamento.</t>
-  </si>
-  <si>
-    <t>Captura-1-Departamentos-fallida.png</t>
-  </si>
-  <si>
-    <t>Código: 2 - Nombre: Departamento QA-Auto 2</t>
-  </si>
-  <si>
-    <t>Captura-2-Departamentos-fallida.png</t>
   </si>
 </sst>
 </file>
@@ -86,7 +65,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -96,11 +75,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0070C0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -116,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -127,7 +101,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,14 +484,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:F7"/>
+  <dimension ref="A2:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
     <col min="3" max="3" width="52" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="79" customWidth="1"/>
+    <col min="5" max="5" width="42" customWidth="1"/>
     <col min="6" max="6" width="52" customWidth="1"/>
   </cols>
   <sheetData>
@@ -554,46 +527,6 @@
       </c>
       <c r="F5" s="3" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
-        <v>1</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>2</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
crud Campos adicionales por entidad y metodo comboboxiframe Mejorado y metodo para logo ( pendiente asignar las transacciones y caracteriscticas al arbol)
</commit_message>
<xml_diff>
--- a/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
+++ b/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
   <si>
     <t>Reporte de Resultados de Pruebas Automatizadas</t>
   </si>
   <si>
-    <t>Generado: 26/3/2026, 14:32:28</t>
+    <t>Generado: 26/3/2026, 18:51:26</t>
   </si>
   <si>
     <t>No de prueba</t>
@@ -35,6 +35,39 @@
   </si>
   <si>
     <t>Evidencia</t>
+  </si>
+  <si>
+    <t>Campos Adicionales Por Entidad</t>
+  </si>
+  <si>
+    <t>Caracteristica: Moneda - Tipo: undefined</t>
+  </si>
+  <si>
+    <t>fallida</t>
+  </si>
+  <si>
+    <t>CASTV-0229 - Error. La caracteristica seleccionada ya esta asignada a la entidad.</t>
+  </si>
+  <si>
+    <t>Captura-1-Campos Adicionales Por Entidad-fallida.png</t>
+  </si>
+  <si>
+    <t>Caracteristica: Efectivo físico - Tipo: undefined</t>
+  </si>
+  <si>
+    <t>exitosa</t>
+  </si>
+  <si>
+    <t>El registro se ha guardado correctamente</t>
+  </si>
+  <si>
+    <t>Captura-2-Campos Adicionales Por Entidad-exitosa.png</t>
+  </si>
+  <si>
+    <t>Caracteristica: Nombre de cliente - Tipo: undefined</t>
+  </si>
+  <si>
+    <t>Captura-3-Campos Adicionales Por Entidad-exitosa.png</t>
   </si>
 </sst>
 </file>
@@ -65,7 +98,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -75,6 +108,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0070C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -101,6 +139,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -484,15 +523,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:F5"/>
+  <dimension ref="A2:F9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="27" customWidth="1"/>
-    <col min="3" max="3" width="52" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="53" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
-    <col min="6" max="6" width="52" customWidth="1"/>
+    <col min="5" max="5" width="80" customWidth="1"/>
+    <col min="6" max="6" width="54" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
@@ -527,6 +566,86 @@
       </c>
       <c r="F5" s="3" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>1</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>2</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
asignar las transacciones individuales pendiente flujo si ya estan asigandas y asignar todas y agregar campos adicionales, se mejora metodo ingreso fecha y agregan metodos para ingresar al arbnol deseado y asignar tx individuales
</commit_message>
<xml_diff>
--- a/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
+++ b/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Reporte de Resultados de Pruebas Automatizadas</t>
   </si>
   <si>
-    <t>Generado: 26/3/2026, 18:51:26</t>
+    <t>Generado: 26/3/2026, 20:24:17</t>
   </si>
   <si>
     <t>No de prueba</t>
@@ -35,39 +35,6 @@
   </si>
   <si>
     <t>Evidencia</t>
-  </si>
-  <si>
-    <t>Campos Adicionales Por Entidad</t>
-  </si>
-  <si>
-    <t>Caracteristica: Moneda - Tipo: undefined</t>
-  </si>
-  <si>
-    <t>fallida</t>
-  </si>
-  <si>
-    <t>CASTV-0229 - Error. La caracteristica seleccionada ya esta asignada a la entidad.</t>
-  </si>
-  <si>
-    <t>Captura-1-Campos Adicionales Por Entidad-fallida.png</t>
-  </si>
-  <si>
-    <t>Caracteristica: Efectivo físico - Tipo: undefined</t>
-  </si>
-  <si>
-    <t>exitosa</t>
-  </si>
-  <si>
-    <t>El registro se ha guardado correctamente</t>
-  </si>
-  <si>
-    <t>Captura-2-Campos Adicionales Por Entidad-exitosa.png</t>
-  </si>
-  <si>
-    <t>Caracteristica: Nombre de cliente - Tipo: undefined</t>
-  </si>
-  <si>
-    <t>Captura-3-Campos Adicionales Por Entidad-exitosa.png</t>
   </si>
 </sst>
 </file>
@@ -98,7 +65,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -108,11 +75,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0070C0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -128,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -139,7 +101,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -523,15 +484,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:F9"/>
+  <dimension ref="A2:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="3" max="3" width="53" customWidth="1"/>
+    <col min="2" max="2" width="27" customWidth="1"/>
+    <col min="3" max="3" width="52" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="80" customWidth="1"/>
-    <col min="6" max="6" width="54" customWidth="1"/>
+    <col min="5" max="5" width="42" customWidth="1"/>
+    <col min="6" max="6" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
@@ -566,86 +527,6 @@
       </c>
       <c r="F5" s="3" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
-        <v>1</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4">
-        <v>2</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ultimos ajustes y creacion de coleccion implementacion
</commit_message>
<xml_diff>
--- a/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
+++ b/ReporteXlsx/ReportePruebasEjecutas-ConfiguracionesIniciales.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="53">
   <si>
     <t>Reporte de Resultados de Pruebas Automatizadas</t>
   </si>
   <si>
-    <t>Generado: 27/3/2026, 19:40:27</t>
+    <t>Generado: 8/4/2026, 15:47:01</t>
   </si>
   <si>
     <t>No de prueba</t>
@@ -35,6 +35,141 @@
   </si>
   <si>
     <t>Evidencia</t>
+  </si>
+  <si>
+    <t>Asignación Característica-Paso</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 1 - Característica: Cuenta</t>
+  </si>
+  <si>
+    <t>exitosa</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Captura-44-AsignacionCaracteristica-exitosa.png</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 1 - Característica: Numero de Tarjeta</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 1 - Característica: Monto</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 1 - Característica: Tipo de ID</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 1 - Característica: N° Identificación</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 2 - Característica: Cuenta</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 2 - Característica: Numero de Tarjeta</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 2 - Característica: Nombre del titular</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 2 - Característica: Moneda</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 2 - Característica: Tipo de producto</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 2 - Característica: Monto</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 2 - Característica: Referencia estado/cuenta</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 2 - Característica: Tipo de ID</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 2 - Característica: N° Identificación</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 2 - Característica: Nombre</t>
+  </si>
+  <si>
+    <t>fallida</t>
+  </si>
+  <si>
+    <t>Captura-44-AsignacionCaracteristica-fallida.png</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 3 - Característica: Moneda</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 3 - Característica: Monto</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 3 - Característica: Monto Cobro TSP</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 3 - Característica: Monto Total</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 3 - Característica: Posee libreta</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 3 - Característica: Efectivo</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 3 - Característica: Efectivo electrónico</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 3 - Característica: Rubro</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Cuenta</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Número de tarjeta</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Nombre del titular</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Referencia estado/cuenta</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Moneda</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Monto</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Monto Cobro TSP</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Monto Total</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Tipo de ID</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: N° Identificación</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Nombre</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Posee libreta</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Efectivo</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Efectivo electrónico</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Rubro</t>
+  </si>
+  <si>
+    <t>Transacción: 1600 - Paso: Paso 4 - Característica: Requiere llenar AML</t>
   </si>
 </sst>
 </file>
@@ -65,7 +200,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -75,6 +210,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0070C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -101,6 +241,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -484,12 +625,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:F5"/>
+  <dimension ref="A2:F44"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="27" customWidth="1"/>
-    <col min="3" max="3" width="52" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="77" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
     <col min="5" max="5" width="42" customWidth="1"/>
     <col min="6" max="6" width="52" customWidth="1"/>
@@ -527,6 +668,786 @@
       </c>
       <c r="F5" s="3" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>44</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>44</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>44</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>44</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>44</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>44</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>44</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>44</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>44</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>44</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>44</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>44</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>44</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>44</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="4">
+        <v>44</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>44</v>
+      </c>
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="4">
+        <v>44</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>44</v>
+      </c>
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="4">
+        <v>44</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>44</v>
+      </c>
+      <c r="B25" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" t="s">
+        <v>33</v>
+      </c>
+      <c r="D25" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="4">
+        <v>44</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>44</v>
+      </c>
+      <c r="B27" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D27" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="4">
+        <v>44</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>44</v>
+      </c>
+      <c r="B29" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="4">
+        <v>44</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>44</v>
+      </c>
+      <c r="B31" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" t="s">
+        <v>39</v>
+      </c>
+      <c r="D31" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="4">
+        <v>44</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>44</v>
+      </c>
+      <c r="B33" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" t="s">
+        <v>41</v>
+      </c>
+      <c r="D33" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="4">
+        <v>44</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>44</v>
+      </c>
+      <c r="B35" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35" t="s">
+        <v>43</v>
+      </c>
+      <c r="D35" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="4">
+        <v>44</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>44</v>
+      </c>
+      <c r="B37" t="s">
+        <v>8</v>
+      </c>
+      <c r="C37" t="s">
+        <v>45</v>
+      </c>
+      <c r="D37" t="s">
+        <v>10</v>
+      </c>
+      <c r="E37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="4">
+        <v>44</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>44</v>
+      </c>
+      <c r="B39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39" t="s">
+        <v>47</v>
+      </c>
+      <c r="D39" t="s">
+        <v>27</v>
+      </c>
+      <c r="E39" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="4">
+        <v>44</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>44</v>
+      </c>
+      <c r="B41" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" t="s">
+        <v>49</v>
+      </c>
+      <c r="D41" t="s">
+        <v>27</v>
+      </c>
+      <c r="E41" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="4">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>44</v>
+      </c>
+      <c r="B43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" t="s">
+        <v>51</v>
+      </c>
+      <c r="D43" t="s">
+        <v>27</v>
+      </c>
+      <c r="E43" t="s">
+        <v>11</v>
+      </c>
+      <c r="F43" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="4">
+        <v>44</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>